<commit_message>
Record verified production release
</commit_message>
<xml_diff>
--- a/documentation/AITSM_Master_Checklist.xlsx
+++ b/documentation/AITSM_Master_Checklist.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Checklist" sheetId="1" r:id="Rd9128dd54e0f4e21"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Checklist" sheetId="1" r:id="R9b8d78e0b334464a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -166,21 +166,12 @@
     <x:t xml:space="preserve">Final public-repository review for historical sensitive data and configuration.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">No open GitHub secret-scanning, Dependabot, or code-scanning alerts.</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">SEC-08</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Focused review of authentication, collector enrollment, uploads, and AI Bridge.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Blocked</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Close after a successful production candidate; review found the legacy production-schema issue.</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Quality Assurance</x:t>
   </x:si>
   <x:si>
@@ -241,43 +232,34 @@
     <x:t xml:space="preserve">Approve production deployment.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Owner approval and protected deployment approval recorded.</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">PROD-06</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Production smoke test.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Wait for successful migration and production promotion.</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">PROD-07</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Confirm rollback revision availability.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Wait for successful production promotion.</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">PROD-08</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Remove legacy Gemini provider/key configuration from production and apply the Beta Ollama/fallback configuration.</x:t>
   </x:si>
   <x:si>
+    <x:t xml:space="preserve">Operations</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">OPS-01</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Document and verify the production database restoration procedure.</x:t>
+  </x:si>
+  <x:si>
     <x:t xml:space="preserve">In progress</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Operations</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">OPS-01</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Document and verify the production database restoration procedure.</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Temporary restore drill is approved and will run after successful release completion.</x:t>
@@ -1105,7 +1087,7 @@
       </x:c>
       <x:c r="D31" s="7"/>
     </x:row>
-    <x:row r="32" ht="15" customHeight="1">
+    <x:row r="32" ht="36" hidden="0" customHeight="1">
       <x:c r="A32" s="4" t="s">
         <x:v>50</x:v>
       </x:c>
@@ -1115,93 +1097,93 @@
       <x:c r="C32" s="6" t="s">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="D32" s="7" t="s">
+      <x:c r="D32" s="18" t="str">
+        <x:v>Public main source, remote branch names, recent commit messages, releases, and deployment metadata were reviewed; no unwanted branding or open GitHub security alerts remain.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="36" hidden="0" customHeight="1">
+      <x:c r="A33" s="4" t="s">
         <x:v>52</x:v>
       </x:c>
-    </x:row>
-    <x:row r="33" ht="24" customHeight="1">
-      <x:c r="A33" s="4" t="s">
+      <x:c r="B33" s="5" t="s">
         <x:v>53</x:v>
       </x:c>
-      <x:c r="B33" s="5" t="s">
-        <x:v>54</x:v>
-      </x:c>
-      <x:c r="C33" s="6" t="s">
-        <x:v>55</x:v>
-      </x:c>
-      <x:c r="D33" s="7" t="s">
-        <x:v>56</x:v>
+      <x:c r="C33" s="6" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="D33" s="18" t="str">
+        <x:v>Focused production review completed. Protected tests, dependency and secret scans, and CodeQL passed; migration compatibility and legacy secret removal were remediated before promotion.</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="15" customHeight="1">
       <x:c r="A34" s="14" t="s">
-        <x:v>57</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="B34" s="15"/>
       <x:c r="C34" s="16"/>
-      <x:c r="D34" s="17"/>
+      <x:c r="D34" s="19"/>
     </x:row>
     <x:row r="35" ht="15" customHeight="1">
       <x:c r="A35" s="4" t="s">
-        <x:v>58</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="B35" s="5" t="s">
-        <x:v>59</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="C35" s="6" t="s">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="D35" s="7"/>
+      <x:c r="D35" s="18"/>
     </x:row>
     <x:row r="36" ht="15" customHeight="1">
       <x:c r="A36" s="4" t="s">
-        <x:v>60</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="B36" s="5" t="s">
-        <x:v>61</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="C36" s="6" t="s">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="D36" s="7"/>
+      <x:c r="D36" s="18"/>
     </x:row>
     <x:row r="37" ht="15" customHeight="1">
       <x:c r="A37" s="14" t="s">
-        <x:v>62</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="B37" s="15"/>
       <x:c r="C37" s="16"/>
-      <x:c r="D37" s="17"/>
+      <x:c r="D37" s="19"/>
     </x:row>
     <x:row r="38" ht="15" customHeight="1">
       <x:c r="A38" s="4" t="s">
-        <x:v>63</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="B38" s="5" t="s">
-        <x:v>64</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="C38" s="6" t="s">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="D38" s="7"/>
+      <x:c r="D38" s="18"/>
     </x:row>
     <x:row r="39" ht="36" hidden="0" customHeight="1">
       <x:c r="A39" s="4" t="s">
-        <x:v>65</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="B39" s="5" t="s">
-        <x:v>66</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="C39" s="6" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D39" s="18" t="str">
-        <x:v>Clean-repository Beta deployment verified on revision aitsm-beta-00042-ver. Health returned HTTP 200 and rollback protection remains active.</x:v>
+        <x:v>Clean-repository Beta deployment verified on final revision aitsm-beta-00044-bes. Health returned HTTP 200, legacy Gemini configuration was absent, and rollback protection remained active.</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="15" customHeight="1">
       <x:c r="A40" s="14" t="s">
-        <x:v>67</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="B40" s="15"/>
       <x:c r="C40" s="16"/>
@@ -1209,105 +1191,105 @@
     </x:row>
     <x:row r="41" ht="15" customHeight="1">
       <x:c r="A41" s="4" t="s">
-        <x:v>68</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="B41" s="5" t="s">
-        <x:v>69</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="C41" s="6" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D41" s="18" t="s">
-        <x:v>70</x:v>
+        <x:v>67</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="36" hidden="0" customHeight="1">
       <x:c r="A42" s="4" t="s">
-        <x:v>71</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="B42" s="5" t="s">
-        <x:v>72</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="C42" s="6" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D42" s="18" t="str">
-        <x:v>Security and deployment run 39451199264 passed. Beta revision aitsm-beta-00042-ver returned HTTP 200 with zero legacy Gemini environment variables.</x:v>
+        <x:v>Final Beta security and deployment run 39454166237 passed. Revision aitsm-beta-00044-bes returned HTTP 200 with zero legacy Gemini environment variables.</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="24" hidden="0" customHeight="1">
       <x:c r="A43" s="4" t="s">
+        <x:v>70</x:v>
+      </x:c>
+      <x:c r="B43" s="5" t="s">
+        <x:v>71</x:v>
+      </x:c>
+      <x:c r="C43" s="6" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="D43" s="18" t="str">
+        <x:v>Protected release PR #5 was merged from beta to main after the verified Beta deployment.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="24" hidden="0" customHeight="1">
+      <x:c r="A44" s="4" t="s">
+        <x:v>72</x:v>
+      </x:c>
+      <x:c r="B44" s="5" t="s">
         <x:v>73</x:v>
       </x:c>
-      <x:c r="B43" s="5" t="s">
+      <x:c r="C44" s="6" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="D44" s="18" t="str">
+        <x:v>Protected production deployment approval was recorded after all required security checks passed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="36" hidden="0" customHeight="1">
+      <x:c r="A45" s="4" t="s">
         <x:v>74</x:v>
       </x:c>
-      <x:c r="C43" s="6" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="D43" s="18" t="str">
-        <x:v>Clean release PR #5 opened from beta to main after the verified Beta deployment.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="44" ht="15" customHeight="1">
-      <x:c r="A44" s="4" t="s">
+      <x:c r="B45" s="5" t="s">
         <x:v>75</x:v>
       </x:c>
-      <x:c r="B44" s="5" t="s">
+      <x:c r="C45" s="6" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="D45" s="18" t="str">
+        <x:v>Production run 39503798792 passed. Revision aitsm-00048-luf serves 100% of traffic; health and landing-page smoke tests both returned HTTP 200.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="24" hidden="0" customHeight="1">
+      <x:c r="A46" s="4" t="s">
         <x:v>76</x:v>
       </x:c>
-      <x:c r="C44" s="6" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="D44" s="18" t="s">
+      <x:c r="B46" s="5" t="s">
         <x:v>77</x:v>
       </x:c>
-    </x:row>
-    <x:row r="45" ht="15" customHeight="1">
-      <x:c r="A45" s="4" t="s">
+      <x:c r="C46" s="6" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="D46" s="18" t="str">
+        <x:v>Previous live revision aitsm-00035-fz5 remains Ready and available as the verified rollback target.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="36" hidden="0" customHeight="1">
+      <x:c r="A47" s="4" t="s">
         <x:v>78</x:v>
       </x:c>
-      <x:c r="B45" s="5" t="s">
+      <x:c r="B47" s="5" t="s">
         <x:v>79</x:v>
       </x:c>
-      <x:c r="C45" s="6" t="s">
-        <x:v>55</x:v>
-      </x:c>
-      <x:c r="D45" s="18" t="s">
-        <x:v>80</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="46" ht="15" customHeight="1">
-      <x:c r="A46" s="4" t="s">
-        <x:v>81</x:v>
-      </x:c>
-      <x:c r="B46" s="5" t="s">
-        <x:v>82</x:v>
-      </x:c>
-      <x:c r="C46" s="6" t="s">
-        <x:v>55</x:v>
-      </x:c>
-      <x:c r="D46" s="18" t="s">
-        <x:v>83</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="47" ht="24" hidden="0" customHeight="1">
-      <x:c r="A47" s="4" t="s">
-        <x:v>84</x:v>
-      </x:c>
-      <x:c r="B47" s="5" t="s">
-        <x:v>85</x:v>
-      </x:c>
-      <x:c r="C47" s="6" t="s">
-        <x:v>86</x:v>
+      <x:c r="C47" s="6" t="str">
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="D47" s="18" t="str">
-        <x:v>Clean Beta is verified. Production remains on the existing healthy revision while PR #5 proceeds through the protected candidate workflow.</x:v>
+        <x:v>Production revision aitsm-00048-luf contains OLLAMA_MODEL=qwen3:8b and zero AI_PROVIDER, GEMINI_MODEL, or GEMINI_API_KEY variables.</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="15" customHeight="1">
       <x:c r="A48" s="14" t="s">
-        <x:v>87</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="B48" s="15"/>
       <x:c r="C48" s="16"/>
@@ -1315,49 +1297,49 @@
     </x:row>
     <x:row r="49" ht="24" customHeight="1">
       <x:c r="A49" s="4" t="s">
-        <x:v>88</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="B49" s="5" t="s">
-        <x:v>89</x:v>
+        <x:v>82</x:v>
       </x:c>
       <x:c r="C49" s="6" t="s">
-        <x:v>86</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="D49" s="7" t="s">
-        <x:v>90</x:v>
+        <x:v>84</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="15" customHeight="1">
       <x:c r="A50" s="4" t="s">
-        <x:v>91</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="B50" s="5" t="s">
-        <x:v>92</x:v>
+        <x:v>86</x:v>
       </x:c>
       <x:c r="C50" s="6" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D50" s="7" t="s">
-        <x:v>93</x:v>
+        <x:v>87</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="15" customHeight="1">
       <x:c r="A51" s="4" t="s">
-        <x:v>94</x:v>
+        <x:v>88</x:v>
       </x:c>
       <x:c r="B51" s="5" t="s">
-        <x:v>95</x:v>
+        <x:v>89</x:v>
       </x:c>
       <x:c r="C51" s="6" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D51" s="7" t="s">
-        <x:v>96</x:v>
+        <x:v>90</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="15" customHeight="1">
       <x:c r="A52" s="14" t="s">
-        <x:v>97</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="B52" s="15"/>
       <x:c r="C52" s="16"/>
@@ -1365,10 +1347,10 @@
     </x:row>
     <x:row r="53" ht="15" customHeight="1">
       <x:c r="A53" s="8" t="s">
-        <x:v>98</x:v>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="B53" s="9" t="s">
-        <x:v>99</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="C53" s="10" t="s">
         <x:v>10</x:v>

</xml_diff>

<commit_message>
Record successful database restore drill
</commit_message>
<xml_diff>
--- a/documentation/AITSM_Master_Checklist.xlsx
+++ b/documentation/AITSM_Master_Checklist.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Checklist" sheetId="1" r:id="R9b8d78e0b334464a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Checklist" sheetId="1" r:id="Raf4c4602c550444d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -257,12 +257,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Document and verify the production database restoration procedure.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">In progress</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Temporary restore drill is approved and will run after successful release completion.</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">OPS-02</x:t>
@@ -1295,51 +1289,51 @@
       <x:c r="C48" s="16"/>
       <x:c r="D48" s="17"/>
     </x:row>
-    <x:row r="49" ht="24" customHeight="1">
+    <x:row r="49" ht="60" hidden="0" customHeight="1">
       <x:c r="A49" s="4" t="s">
         <x:v>81</x:v>
       </x:c>
       <x:c r="B49" s="5" t="s">
         <x:v>82</x:v>
       </x:c>
-      <x:c r="C49" s="6" t="s">
-        <x:v>83</x:v>
-      </x:c>
-      <x:c r="D49" s="7" t="s">
-        <x:v>84</x:v>
+      <x:c r="C49" s="6" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="D49" s="18" t="str">
+        <x:v>Backup 1792325031222 was restored to temporary PostgreSQL 16 instance aitsm-restore-drill-20261021. The instance was RUNNABLE, the restored production database exposed 27 public tables, and read-only users/tickets queries succeeded. The temporary instance was deleted; production and the backup remain healthy.</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="15" customHeight="1">
       <x:c r="A50" s="4" t="s">
+        <x:v>83</x:v>
+      </x:c>
+      <x:c r="B50" s="5" t="s">
+        <x:v>84</x:v>
+      </x:c>
+      <x:c r="C50" s="6" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="D50" s="7" t="s">
         <x:v>85</x:v>
-      </x:c>
-      <x:c r="B50" s="5" t="s">
-        <x:v>86</x:v>
-      </x:c>
-      <x:c r="C50" s="6" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="D50" s="7" t="s">
-        <x:v>87</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="15" customHeight="1">
       <x:c r="A51" s="4" t="s">
+        <x:v>86</x:v>
+      </x:c>
+      <x:c r="B51" s="5" t="s">
+        <x:v>87</x:v>
+      </x:c>
+      <x:c r="C51" s="6" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="D51" s="7" t="s">
         <x:v>88</x:v>
-      </x:c>
-      <x:c r="B51" s="5" t="s">
-        <x:v>89</x:v>
-      </x:c>
-      <x:c r="C51" s="6" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="D51" s="7" t="s">
-        <x:v>90</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="15" customHeight="1">
       <x:c r="A52" s="14" t="s">
-        <x:v>91</x:v>
+        <x:v>89</x:v>
       </x:c>
       <x:c r="B52" s="15"/>
       <x:c r="C52" s="16"/>
@@ -1347,10 +1341,10 @@
     </x:row>
     <x:row r="53" ht="15" customHeight="1">
       <x:c r="A53" s="8" t="s">
-        <x:v>92</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="B53" s="9" t="s">
-        <x:v>93</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="C53" s="10" t="s">
         <x:v>10</x:v>

</xml_diff>

<commit_message>
Update master checklist with Beta hardening results
</commit_message>
<xml_diff>
--- a/documentation/AITSM_Master_Checklist.xlsx
+++ b/documentation/AITSM_Master_Checklist.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Checklist" sheetId="1" r:id="Raf4c4602c550444d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Checklist" sheetId="1" r:id="R09da3c8a255f40b7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -89,9 +89,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Enrollment, telemetry, discovery, refresh, repair, revocation, deduplication, and dynamic-IP support.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Includes two-device acceptance, revoked collector rejection, and dynamic-IP deduplication.</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">COL-19–20</x:t>
@@ -811,7 +808,7 @@
       <x:c r="C6" s="16"/>
       <x:c r="D6" s="17"/>
     </x:row>
-    <x:row r="7" ht="24" customHeight="1">
+    <x:row r="7" ht="76" customHeight="1">
       <x:c r="A7" s="4" t="s">
         <x:v>5</x:v>
       </x:c>
@@ -821,7 +818,9 @@
       <x:c r="C7" s="6" t="s">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="D7" s="7"/>
+      <x:c r="D7" s="7" t="str">
+        <x:v>Beta hardening completed: only Super Admin can grant or revoke administrator roles, manage administrator accounts, or change system security settings. Backend authorization blocks direct API bypass. Temporary-password accounts must replace the password before protected access.</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="15" customHeight="1">
       <x:c r="A8" s="4" t="s">
@@ -843,7 +842,7 @@
       <x:c r="C9" s="16"/>
       <x:c r="D9" s="17"/>
     </x:row>
-    <x:row r="10" ht="24" customHeight="1">
+    <x:row r="10" ht="86" customHeight="1">
       <x:c r="A10" s="4" t="s">
         <x:v>12</x:v>
       </x:c>
@@ -853,7 +852,9 @@
       <x:c r="C10" s="6" t="s">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="D10" s="7"/>
+      <x:c r="D10" s="7" t="str">
+        <x:v>Beta hardening completed: user-scoped counters now separate Open, In Progress, Resolved, Closed, and Total. Backend rules enforce Open → In Progress → Resolved → Closed and Resolved → In Progress. Resolution notes, history, and secure authenticated PNG/JPEG/WebP attachments are preserved.</x:v>
+      </x:c>
     </x:row>
     <x:row r="11" ht="15" customHeight="1">
       <x:c r="A11" s="14" t="s">
@@ -927,7 +928,7 @@
       <x:c r="C17" s="16"/>
       <x:c r="D17" s="17"/>
     </x:row>
-    <x:row r="18" ht="24" customHeight="1">
+    <x:row r="18" ht="88" customHeight="1">
       <x:c r="A18" s="4" t="s">
         <x:v>25</x:v>
       </x:c>
@@ -937,16 +938,16 @@
       <x:c r="C18" s="6" t="s">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="D18" s="7" t="s">
-        <x:v>27</x:v>
+      <x:c r="D18" s="7" t="str">
+        <x:v>Includes two-device acceptance, revoked collector rejection, and dynamic-IP deduplication. The collector release remains HTTPS-hosted, SHA-256-pinned, scope-authorized, and free of localhost or machine-specific paths. Automated portability checks passed; a separate-PC install remains a manual acceptance test.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="15" customHeight="1">
       <x:c r="A19" s="4" t="s">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="B19" s="5" t="s">
         <x:v>28</x:v>
-      </x:c>
-      <x:c r="B19" s="5" t="s">
-        <x:v>29</x:v>
       </x:c>
       <x:c r="C19" s="6" t="s">
         <x:v>10</x:v>
@@ -955,7 +956,7 @@
     </x:row>
     <x:row r="20" ht="15" customHeight="1">
       <x:c r="A20" s="14" t="s">
-        <x:v>30</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="B20" s="15"/>
       <x:c r="C20" s="16"/>
@@ -963,10 +964,10 @@
     </x:row>
     <x:row r="21" ht="24" customHeight="1">
       <x:c r="A21" s="4" t="s">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="B21" s="5" t="s">
         <x:v>31</x:v>
-      </x:c>
-      <x:c r="B21" s="5" t="s">
-        <x:v>32</x:v>
       </x:c>
       <x:c r="C21" s="6" t="s">
         <x:v>7</x:v>
@@ -975,7 +976,7 @@
     </x:row>
     <x:row r="22" ht="15" customHeight="1">
       <x:c r="A22" s="14" t="s">
-        <x:v>33</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="B22" s="15"/>
       <x:c r="C22" s="16"/>
@@ -983,10 +984,10 @@
     </x:row>
     <x:row r="23" ht="15" customHeight="1">
       <x:c r="A23" s="4" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="B23" s="5" t="s">
         <x:v>34</x:v>
-      </x:c>
-      <x:c r="B23" s="5" t="s">
-        <x:v>35</x:v>
       </x:c>
       <x:c r="C23" s="6" t="s">
         <x:v>7</x:v>
@@ -995,7 +996,7 @@
     </x:row>
     <x:row r="24" ht="15" customHeight="1">
       <x:c r="A24" s="14" t="s">
-        <x:v>36</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="B24" s="15"/>
       <x:c r="C24" s="16"/>
@@ -1003,10 +1004,10 @@
     </x:row>
     <x:row r="25" ht="15" customHeight="1">
       <x:c r="A25" s="4" t="s">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="B25" s="5" t="s">
         <x:v>37</x:v>
-      </x:c>
-      <x:c r="B25" s="5" t="s">
-        <x:v>38</x:v>
       </x:c>
       <x:c r="C25" s="6" t="s">
         <x:v>7</x:v>
@@ -1015,10 +1016,10 @@
     </x:row>
     <x:row r="26" ht="15" customHeight="1">
       <x:c r="A26" s="4" t="s">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="B26" s="5" t="s">
         <x:v>39</x:v>
-      </x:c>
-      <x:c r="B26" s="5" t="s">
-        <x:v>40</x:v>
       </x:c>
       <x:c r="C26" s="6" t="s">
         <x:v>10</x:v>
@@ -1027,10 +1028,10 @@
     </x:row>
     <x:row r="27" ht="15" customHeight="1">
       <x:c r="A27" s="4" t="s">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="B27" s="5" t="s">
         <x:v>41</x:v>
-      </x:c>
-      <x:c r="B27" s="5" t="s">
-        <x:v>42</x:v>
       </x:c>
       <x:c r="C27" s="6" t="s">
         <x:v>7</x:v>
@@ -1039,10 +1040,10 @@
     </x:row>
     <x:row r="28" ht="15" customHeight="1">
       <x:c r="A28" s="4" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="B28" s="5" t="s">
         <x:v>43</x:v>
-      </x:c>
-      <x:c r="B28" s="5" t="s">
-        <x:v>44</x:v>
       </x:c>
       <x:c r="C28" s="6" t="s">
         <x:v>7</x:v>
@@ -1051,10 +1052,10 @@
     </x:row>
     <x:row r="29" ht="15" customHeight="1">
       <x:c r="A29" s="4" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="B29" s="5" t="s">
         <x:v>45</x:v>
-      </x:c>
-      <x:c r="B29" s="5" t="s">
-        <x:v>46</x:v>
       </x:c>
       <x:c r="C29" s="6" t="s">
         <x:v>10</x:v>
@@ -1063,7 +1064,7 @@
     </x:row>
     <x:row r="30" ht="15" customHeight="1">
       <x:c r="A30" s="14" t="s">
-        <x:v>47</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="B30" s="15"/>
       <x:c r="C30" s="16"/>
@@ -1071,10 +1072,10 @@
     </x:row>
     <x:row r="31" ht="15" customHeight="1">
       <x:c r="A31" s="4" t="s">
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="B31" s="5" t="s">
         <x:v>48</x:v>
-      </x:c>
-      <x:c r="B31" s="5" t="s">
-        <x:v>49</x:v>
       </x:c>
       <x:c r="C31" s="6" t="s">
         <x:v>7</x:v>
@@ -1083,10 +1084,10 @@
     </x:row>
     <x:row r="32" ht="36" hidden="0" customHeight="1">
       <x:c r="A32" s="4" t="s">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="B32" s="5" t="s">
         <x:v>50</x:v>
-      </x:c>
-      <x:c r="B32" s="5" t="s">
-        <x:v>51</x:v>
       </x:c>
       <x:c r="C32" s="6" t="s">
         <x:v>7</x:v>
@@ -1095,46 +1096,48 @@
         <x:v>Public main source, remote branch names, recent commit messages, releases, and deployment metadata were reviewed; no unwanted branding or open GitHub security alerts remain.</x:v>
       </x:c>
     </x:row>
-    <x:row r="33" ht="36" hidden="0" customHeight="1">
+    <x:row r="33" ht="72" hidden="0" customHeight="1">
       <x:c r="A33" s="4" t="s">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="B33" s="5" t="s">
         <x:v>52</x:v>
-      </x:c>
-      <x:c r="B33" s="5" t="s">
-        <x:v>53</x:v>
       </x:c>
       <x:c r="C33" s="6" t="str">
         <x:v>Done</x:v>
       </x:c>
       <x:c r="D33" s="18" t="str">
-        <x:v>Focused production review completed. Protected tests, dependency and secret scans, and CodeQL passed; migration compatibility and legacy secret removal were remediated before promotion.</x:v>
+        <x:v>Focused production review completed. Protected tests, dependency and secret scans, and CodeQL passed. The new RBAC boundaries, attachment authorization, image decoding, and mandatory-password middleware also passed protected review on PR #9.</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="15" customHeight="1">
       <x:c r="A34" s="14" t="s">
-        <x:v>54</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="B34" s="15"/>
       <x:c r="C34" s="16"/>
       <x:c r="D34" s="19"/>
     </x:row>
-    <x:row r="35" ht="15" customHeight="1">
+    <x:row r="35" ht="92" customHeight="1">
       <x:c r="A35" s="4" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="B35" s="5" t="s">
         <x:v>55</x:v>
       </x:c>
-      <x:c r="B35" s="5" t="s">
-        <x:v>56</x:v>
-      </x:c>
       <x:c r="C35" s="6" t="s">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="D35" s="18"/>
+      <x:c r="D35" s="18" t="str">
+        <x:v>111 automated tests passed. JavaScript syntax, dependency scanning with zero reported vulnerabilities, secret scanning, and Java/Kotlin and JavaScript CodeQL passed. Beta smoke tests returned HTTP 200. Manual acceptance remains for the two-role UI, browser attachment flow, forced-password flow, and separate-PC collector installation.</x:v>
+      </x:c>
     </x:row>
     <x:row r="36" ht="15" customHeight="1">
       <x:c r="A36" s="4" t="s">
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="B36" s="5" t="s">
         <x:v>57</x:v>
-      </x:c>
-      <x:c r="B36" s="5" t="s">
-        <x:v>58</x:v>
       </x:c>
       <x:c r="C36" s="6" t="s">
         <x:v>10</x:v>
@@ -1143,7 +1146,7 @@
     </x:row>
     <x:row r="37" ht="15" customHeight="1">
       <x:c r="A37" s="14" t="s">
-        <x:v>59</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="B37" s="15"/>
       <x:c r="C37" s="16"/>
@@ -1151,33 +1154,33 @@
     </x:row>
     <x:row r="38" ht="15" customHeight="1">
       <x:c r="A38" s="4" t="s">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="B38" s="5" t="s">
         <x:v>60</x:v>
       </x:c>
-      <x:c r="B38" s="5" t="s">
+      <x:c r="C38" s="6" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="D38" s="18"/>
+    </x:row>
+    <x:row r="39" ht="76" hidden="0" customHeight="1">
+      <x:c r="A39" s="4" t="s">
         <x:v>61</x:v>
       </x:c>
-      <x:c r="C38" s="6" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="D38" s="18"/>
-    </x:row>
-    <x:row r="39" ht="36" hidden="0" customHeight="1">
-      <x:c r="A39" s="4" t="s">
+      <x:c r="B39" s="5" t="s">
         <x:v>62</x:v>
       </x:c>
-      <x:c r="B39" s="5" t="s">
-        <x:v>63</x:v>
-      </x:c>
       <x:c r="C39" s="6" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D39" s="18" t="str">
-        <x:v>Clean-repository Beta deployment verified on final revision aitsm-beta-00044-bes. Health returned HTTP 200, legacy Gemini configuration was absent, and rollback protection remained active.</x:v>
+        <x:v>Six-issue Beta hardening is live on revision aitsm-beta-00052-waz from commit 569d2aa12b684ee9bdc4a084427430fedb4c0323. Three post-promotion health checks returned HTTP 200, legacy Gemini variables remain absent, and the prior revision is retained for rollback.</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="15" customHeight="1">
       <x:c r="A40" s="14" t="s">
-        <x:v>64</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="B40" s="15"/>
       <x:c r="C40" s="16"/>
@@ -1185,24 +1188,24 @@
     </x:row>
     <x:row r="41" ht="15" customHeight="1">
       <x:c r="A41" s="4" t="s">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="B41" s="5" t="s">
         <x:v>65</x:v>
       </x:c>
-      <x:c r="B41" s="5" t="s">
+      <x:c r="C41" s="6" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="D41" s="18" t="s">
         <x:v>66</x:v>
-      </x:c>
-      <x:c r="C41" s="6" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="D41" s="18" t="s">
-        <x:v>67</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="36" hidden="0" customHeight="1">
       <x:c r="A42" s="4" t="s">
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="B42" s="5" t="s">
         <x:v>68</x:v>
-      </x:c>
-      <x:c r="B42" s="5" t="s">
-        <x:v>69</x:v>
       </x:c>
       <x:c r="C42" s="6" t="s">
         <x:v>7</x:v>
@@ -1213,10 +1216,10 @@
     </x:row>
     <x:row r="43" ht="24" hidden="0" customHeight="1">
       <x:c r="A43" s="4" t="s">
+        <x:v>69</x:v>
+      </x:c>
+      <x:c r="B43" s="5" t="s">
         <x:v>70</x:v>
-      </x:c>
-      <x:c r="B43" s="5" t="s">
-        <x:v>71</x:v>
       </x:c>
       <x:c r="C43" s="6" t="s">
         <x:v>7</x:v>
@@ -1227,10 +1230,10 @@
     </x:row>
     <x:row r="44" ht="24" hidden="0" customHeight="1">
       <x:c r="A44" s="4" t="s">
+        <x:v>71</x:v>
+      </x:c>
+      <x:c r="B44" s="5" t="s">
         <x:v>72</x:v>
-      </x:c>
-      <x:c r="B44" s="5" t="s">
-        <x:v>73</x:v>
       </x:c>
       <x:c r="C44" s="6" t="s">
         <x:v>7</x:v>
@@ -1241,10 +1244,10 @@
     </x:row>
     <x:row r="45" ht="36" hidden="0" customHeight="1">
       <x:c r="A45" s="4" t="s">
+        <x:v>73</x:v>
+      </x:c>
+      <x:c r="B45" s="5" t="s">
         <x:v>74</x:v>
-      </x:c>
-      <x:c r="B45" s="5" t="s">
-        <x:v>75</x:v>
       </x:c>
       <x:c r="C45" s="6" t="str">
         <x:v>Done</x:v>
@@ -1255,10 +1258,10 @@
     </x:row>
     <x:row r="46" ht="24" hidden="0" customHeight="1">
       <x:c r="A46" s="4" t="s">
+        <x:v>75</x:v>
+      </x:c>
+      <x:c r="B46" s="5" t="s">
         <x:v>76</x:v>
-      </x:c>
-      <x:c r="B46" s="5" t="s">
-        <x:v>77</x:v>
       </x:c>
       <x:c r="C46" s="6" t="str">
         <x:v>Done</x:v>
@@ -1269,10 +1272,10 @@
     </x:row>
     <x:row r="47" ht="36" hidden="0" customHeight="1">
       <x:c r="A47" s="4" t="s">
+        <x:v>77</x:v>
+      </x:c>
+      <x:c r="B47" s="5" t="s">
         <x:v>78</x:v>
-      </x:c>
-      <x:c r="B47" s="5" t="s">
-        <x:v>79</x:v>
       </x:c>
       <x:c r="C47" s="6" t="str">
         <x:v>Done</x:v>
@@ -1283,7 +1286,7 @@
     </x:row>
     <x:row r="48" ht="15" customHeight="1">
       <x:c r="A48" s="14" t="s">
-        <x:v>80</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="B48" s="15"/>
       <x:c r="C48" s="16"/>
@@ -1291,10 +1294,10 @@
     </x:row>
     <x:row r="49" ht="60" hidden="0" customHeight="1">
       <x:c r="A49" s="4" t="s">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="B49" s="5" t="s">
         <x:v>81</x:v>
-      </x:c>
-      <x:c r="B49" s="5" t="s">
-        <x:v>82</x:v>
       </x:c>
       <x:c r="C49" s="6" t="str">
         <x:v>Done</x:v>
@@ -1305,35 +1308,35 @@
     </x:row>
     <x:row r="50" ht="15" customHeight="1">
       <x:c r="A50" s="4" t="s">
+        <x:v>82</x:v>
+      </x:c>
+      <x:c r="B50" s="5" t="s">
         <x:v>83</x:v>
       </x:c>
-      <x:c r="B50" s="5" t="s">
+      <x:c r="C50" s="6" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="D50" s="7" t="s">
         <x:v>84</x:v>
-      </x:c>
-      <x:c r="C50" s="6" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="D50" s="7" t="s">
-        <x:v>85</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="15" customHeight="1">
       <x:c r="A51" s="4" t="s">
+        <x:v>85</x:v>
+      </x:c>
+      <x:c r="B51" s="5" t="s">
         <x:v>86</x:v>
       </x:c>
-      <x:c r="B51" s="5" t="s">
+      <x:c r="C51" s="6" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="D51" s="7" t="s">
         <x:v>87</x:v>
-      </x:c>
-      <x:c r="C51" s="6" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="D51" s="7" t="s">
-        <x:v>88</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="15" customHeight="1">
       <x:c r="A52" s="14" t="s">
-        <x:v>89</x:v>
+        <x:v>88</x:v>
       </x:c>
       <x:c r="B52" s="15"/>
       <x:c r="C52" s="16"/>
@@ -1341,10 +1344,10 @@
     </x:row>
     <x:row r="53" ht="15" customHeight="1">
       <x:c r="A53" s="8" t="s">
+        <x:v>89</x:v>
+      </x:c>
+      <x:c r="B53" s="9" t="s">
         <x:v>90</x:v>
-      </x:c>
-      <x:c r="B53" s="9" t="s">
-        <x:v>91</x:v>
       </x:c>
       <x:c r="C53" s="10" t="s">
         <x:v>10</x:v>

</xml_diff>

<commit_message>
Show ticket trend data for single periods
</commit_message>
<xml_diff>
--- a/documentation/AITSM_Master_Checklist.xlsx
+++ b/documentation/AITSM_Master_Checklist.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Checklist" sheetId="1" r:id="R09da3c8a255f40b7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Checklist" sheetId="1" r:id="Re3593da7c94647ad"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -40,63 +40,60 @@
     <x:t xml:space="preserve">Full invite, password-reset, MFA, suspension, and role-change regression pass.</x:t>
   </x:si>
   <x:si>
+    <x:t xml:space="preserve">Ticket Management</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">TKT-01–16</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Ticket creation through closure, notes, requester updates, ownership lock, Super Admin override, and AI restrictions.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Service Level Agreements</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">SLA-01–07</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">24/7 SLA timing, risk scoring, warning alerts, and breach events.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">SLA-08</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Notifications and Operational Feed</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">NTF-01–09</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Live operational feed, multi-admin notifications, pagination, filtering, and retention configuration.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">NTF-10 / QA-16</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Confirm scheduled notification retention cleanup with real elapsed data.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Collectors and Monitoring</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">COL-01–18</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Enrollment, telemetry, discovery, refresh, repair, revocation, deduplication, and dynamic-IP support.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">COL-19–20</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Collector update policy and possible macOS/Linux support.</x:t>
+  </x:si>
+  <x:si>
     <x:t xml:space="preserve">After launch</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Ticket Management</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">TKT-01–16</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Ticket creation through closure, notes, requester updates, ownership lock, Super Admin override, and AI restrictions.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Service Level Agreements</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">SLA-01–07</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">24/7 SLA timing, risk scoring, warning alerts, and breach events.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">SLA-08</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Confirm SLA targets against the official organization support policy.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Notifications and Operational Feed</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">NTF-01–09</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Live operational feed, multi-admin notifications, pagination, filtering, and retention configuration.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">NTF-10 / QA-16</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Confirm scheduled notification retention cleanup with real elapsed data.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Collectors and Monitoring</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">COL-01–18</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Enrollment, telemetry, discovery, refresh, repair, revocation, deduplication, and dynamic-IP support.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">COL-19–20</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Collector update policy and possible macOS/Linux support.</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">AI Assistance</x:t>
   </x:si>
   <x:si>
@@ -127,9 +124,6 @@
     <x:t xml:space="preserve">KB-02</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Add reviewed real troubleshooting articles.</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">COLLAB-01</x:t>
   </x:si>
   <x:si>
@@ -179,9 +173,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">QA-17</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Add browser-level end-to-end regression tests.</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Source Control and Release Engineering</x:t>
@@ -829,14 +820,14 @@
       <x:c r="B8" s="5" t="s">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="C8" s="6" t="s">
-        <x:v>10</x:v>
+      <x:c r="C8" s="6" t="str">
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="D8" s="7"/>
     </x:row>
     <x:row r="9" ht="15" customHeight="1">
       <x:c r="A9" s="14" t="s">
-        <x:v>11</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="B9" s="15"/>
       <x:c r="C9" s="16"/>
@@ -844,10 +835,10 @@
     </x:row>
     <x:row r="10" ht="86" customHeight="1">
       <x:c r="A10" s="4" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B10" s="5" t="s">
         <x:v>12</x:v>
-      </x:c>
-      <x:c r="B10" s="5" t="s">
-        <x:v>13</x:v>
       </x:c>
       <x:c r="C10" s="6" t="s">
         <x:v>7</x:v>
@@ -858,7 +849,7 @@
     </x:row>
     <x:row r="11" ht="15" customHeight="1">
       <x:c r="A11" s="14" t="s">
-        <x:v>14</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="B11" s="15"/>
       <x:c r="C11" s="16"/>
@@ -866,31 +857,33 @@
     </x:row>
     <x:row r="12" ht="15" customHeight="1">
       <x:c r="A12" s="4" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B12" s="5" t="s">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="B12" s="5" t="s">
+      <x:c r="C12" s="6" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="D12" s="7"/>
+    </x:row>
+    <x:row r="13" ht="24" hidden="0" customHeight="1">
+      <x:c r="A13" s="4" t="s">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="C12" s="6" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="D12" s="7"/>
-    </x:row>
-    <x:row r="13" ht="15" customHeight="1">
-      <x:c r="A13" s="4" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="B13" s="5" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="C13" s="6" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="D13" s="7"/>
+      <x:c r="B13" s="5" t="str">
+        <x:v>SLA targets remain configurable by authorized Super Admins in Settings.</x:v>
+      </x:c>
+      <x:c r="C13" s="6" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="D13" s="7" t="str">
+        <x:v>Separate fixed-policy confirmation is not applicable because authorized Super Admins manage SLA targets in the web app.</x:v>
+      </x:c>
     </x:row>
     <x:row r="14" ht="15" customHeight="1">
       <x:c r="A14" s="14" t="s">
-        <x:v>19</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="B14" s="15"/>
       <x:c r="C14" s="16"/>
@@ -898,31 +891,33 @@
     </x:row>
     <x:row r="15" ht="15" customHeight="1">
       <x:c r="A15" s="4" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="B15" s="5" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="C15" s="6" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="D15" s="7"/>
+    </x:row>
+    <x:row r="16" ht="24" hidden="0" customHeight="1">
+      <x:c r="A16" s="4" t="s">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="B15" s="5" t="s">
+      <x:c r="B16" s="5" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="C15" s="6" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="D15" s="7"/>
-    </x:row>
-    <x:row r="16" ht="15" customHeight="1">
-      <x:c r="A16" s="4" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="B16" s="5" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="C16" s="6" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="D16" s="7"/>
+      <x:c r="C16" s="6" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="D16" s="7" t="str">
+        <x:v>User-confirmed retention acceptance passed after Beta was used solely for development and validation.</x:v>
+      </x:c>
     </x:row>
     <x:row r="17" ht="15" customHeight="1">
       <x:c r="A17" s="14" t="s">
-        <x:v>24</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="B17" s="15"/>
       <x:c r="C17" s="16"/>
@@ -930,10 +925,10 @@
     </x:row>
     <x:row r="18" ht="88" customHeight="1">
       <x:c r="A18" s="4" t="s">
-        <x:v>25</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="B18" s="5" t="s">
-        <x:v>26</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="C18" s="6" t="s">
         <x:v>7</x:v>
@@ -944,19 +939,19 @@
     </x:row>
     <x:row r="19" ht="15" customHeight="1">
       <x:c r="A19" s="4" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="B19" s="5" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="C19" s="6" t="s">
         <x:v>27</x:v>
-      </x:c>
-      <x:c r="B19" s="5" t="s">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="C19" s="6" t="s">
-        <x:v>10</x:v>
       </x:c>
       <x:c r="D19" s="7"/>
     </x:row>
     <x:row r="20" ht="15" customHeight="1">
       <x:c r="A20" s="14" t="s">
-        <x:v>29</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="B20" s="15"/>
       <x:c r="C20" s="16"/>
@@ -964,10 +959,10 @@
     </x:row>
     <x:row r="21" ht="24" customHeight="1">
       <x:c r="A21" s="4" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B21" s="5" t="s">
         <x:v>30</x:v>
-      </x:c>
-      <x:c r="B21" s="5" t="s">
-        <x:v>31</x:v>
       </x:c>
       <x:c r="C21" s="6" t="s">
         <x:v>7</x:v>
@@ -976,7 +971,7 @@
     </x:row>
     <x:row r="22" ht="15" customHeight="1">
       <x:c r="A22" s="14" t="s">
-        <x:v>32</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="B22" s="15"/>
       <x:c r="C22" s="16"/>
@@ -984,10 +979,10 @@
     </x:row>
     <x:row r="23" ht="15" customHeight="1">
       <x:c r="A23" s="4" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="B23" s="5" t="s">
         <x:v>33</x:v>
-      </x:c>
-      <x:c r="B23" s="5" t="s">
-        <x:v>34</x:v>
       </x:c>
       <x:c r="C23" s="6" t="s">
         <x:v>7</x:v>
@@ -996,7 +991,7 @@
     </x:row>
     <x:row r="24" ht="15" customHeight="1">
       <x:c r="A24" s="14" t="s">
-        <x:v>35</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="B24" s="15"/>
       <x:c r="C24" s="16"/>
@@ -1004,34 +999,36 @@
     </x:row>
     <x:row r="25" ht="15" customHeight="1">
       <x:c r="A25" s="4" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="B25" s="5" t="s">
         <x:v>36</x:v>
       </x:c>
-      <x:c r="B25" s="5" t="s">
+      <x:c r="C25" s="6" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="D25" s="7"/>
+    </x:row>
+    <x:row r="26" ht="24" hidden="0" customHeight="1">
+      <x:c r="A26" s="4" t="s">
         <x:v>37</x:v>
       </x:c>
-      <x:c r="C25" s="6" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="D25" s="7"/>
-    </x:row>
-    <x:row r="26" ht="15" customHeight="1">
-      <x:c r="A26" s="4" t="s">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="B26" s="5" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="C26" s="6" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="D26" s="7"/>
+      <x:c r="B26" s="5" t="str">
+        <x:v>Automatically detect recurring resolved issues and create a reviewable knowledge-base candidate after three similar occurrences.</x:v>
+      </x:c>
+      <x:c r="C26" s="6" t="str">
+        <x:v>Approved</x:v>
+      </x:c>
+      <x:c r="D26" s="7" t="str">
+        <x:v>Approved design: store the suggested article, category, source ticket IDs, and occurrence count; require Super Admin review before publication.</x:v>
+      </x:c>
     </x:row>
     <x:row r="27" ht="15" customHeight="1">
       <x:c r="A27" s="4" t="s">
-        <x:v>40</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="B27" s="5" t="s">
-        <x:v>41</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="C27" s="6" t="s">
         <x:v>7</x:v>
@@ -1040,31 +1037,33 @@
     </x:row>
     <x:row r="28" ht="15" customHeight="1">
       <x:c r="A28" s="4" t="s">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="B28" s="5" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="C28" s="6" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="D28" s="7"/>
+    </x:row>
+    <x:row r="29" ht="24" hidden="0" customHeight="1">
+      <x:c r="A29" s="4" t="s">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="B28" s="5" t="s">
+      <x:c r="B29" s="5" t="s">
         <x:v>43</x:v>
       </x:c>
-      <x:c r="C28" s="6" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="D28" s="7"/>
-    </x:row>
-    <x:row r="29" ht="15" customHeight="1">
-      <x:c r="A29" s="4" t="s">
-        <x:v>44</x:v>
-      </x:c>
-      <x:c r="B29" s="5" t="s">
-        <x:v>45</x:v>
-      </x:c>
-      <x:c r="C29" s="6" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="D29" s="7"/>
+      <x:c r="C29" s="6" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="D29" s="7" t="str">
+        <x:v>User-confirmed accessibility, responsive behavior, and Beta feedback checks passed.</x:v>
+      </x:c>
     </x:row>
     <x:row r="30" ht="15" customHeight="1">
       <x:c r="A30" s="14" t="s">
-        <x:v>46</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="B30" s="15"/>
       <x:c r="C30" s="16"/>
@@ -1072,10 +1071,10 @@
     </x:row>
     <x:row r="31" ht="15" customHeight="1">
       <x:c r="A31" s="4" t="s">
-        <x:v>47</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="B31" s="5" t="s">
-        <x:v>48</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="C31" s="6" t="s">
         <x:v>7</x:v>
@@ -1084,10 +1083,10 @@
     </x:row>
     <x:row r="32" ht="36" hidden="0" customHeight="1">
       <x:c r="A32" s="4" t="s">
-        <x:v>49</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="B32" s="5" t="s">
-        <x:v>50</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="C32" s="6" t="s">
         <x:v>7</x:v>
@@ -1098,10 +1097,10 @@
     </x:row>
     <x:row r="33" ht="72" hidden="0" customHeight="1">
       <x:c r="A33" s="4" t="s">
-        <x:v>51</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="B33" s="5" t="s">
-        <x:v>52</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C33" s="6" t="str">
         <x:v>Done</x:v>
@@ -1112,7 +1111,7 @@
     </x:row>
     <x:row r="34" ht="15" customHeight="1">
       <x:c r="A34" s="14" t="s">
-        <x:v>53</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="B34" s="15"/>
       <x:c r="C34" s="16"/>
@@ -1120,10 +1119,10 @@
     </x:row>
     <x:row r="35" ht="92" customHeight="1">
       <x:c r="A35" s="4" t="s">
-        <x:v>54</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="B35" s="5" t="s">
-        <x:v>55</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="C35" s="6" t="s">
         <x:v>7</x:v>
@@ -1132,21 +1131,23 @@
         <x:v>111 automated tests passed. JavaScript syntax, dependency scanning with zero reported vulnerabilities, secret scanning, and Java/Kotlin and JavaScript CodeQL passed. Beta smoke tests returned HTTP 200. Manual acceptance remains for the two-role UI, browser attachment flow, forced-password flow, and separate-PC collector installation.</x:v>
       </x:c>
     </x:row>
-    <x:row r="36" ht="15" customHeight="1">
+    <x:row r="36" ht="14.25" hidden="0" customHeight="1">
       <x:c r="A36" s="4" t="s">
-        <x:v>56</x:v>
-      </x:c>
-      <x:c r="B36" s="5" t="s">
-        <x:v>57</x:v>
-      </x:c>
-      <x:c r="C36" s="6" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="D36" s="18"/>
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="B36" s="5" t="str">
+        <x:v>Browser-level end-to-end regression pass.</x:v>
+      </x:c>
+      <x:c r="C36" s="6" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="D36" s="18" t="str">
+        <x:v>User-confirmed browser-level regression passed.</x:v>
+      </x:c>
     </x:row>
     <x:row r="37" ht="15" customHeight="1">
       <x:c r="A37" s="14" t="s">
-        <x:v>58</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="B37" s="15"/>
       <x:c r="C37" s="16"/>
@@ -1154,10 +1155,10 @@
     </x:row>
     <x:row r="38" ht="15" customHeight="1">
       <x:c r="A38" s="4" t="s">
-        <x:v>59</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="B38" s="5" t="s">
-        <x:v>60</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="C38" s="6" t="s">
         <x:v>7</x:v>
@@ -1166,10 +1167,10 @@
     </x:row>
     <x:row r="39" ht="76" hidden="0" customHeight="1">
       <x:c r="A39" s="4" t="s">
-        <x:v>61</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="B39" s="5" t="s">
-        <x:v>62</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="C39" s="6" t="s">
         <x:v>7</x:v>
@@ -1180,7 +1181,7 @@
     </x:row>
     <x:row r="40" ht="15" customHeight="1">
       <x:c r="A40" s="14" t="s">
-        <x:v>63</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="B40" s="15"/>
       <x:c r="C40" s="16"/>
@@ -1188,24 +1189,24 @@
     </x:row>
     <x:row r="41" ht="15" customHeight="1">
       <x:c r="A41" s="4" t="s">
-        <x:v>64</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="B41" s="5" t="s">
-        <x:v>65</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="C41" s="6" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D41" s="18" t="s">
-        <x:v>66</x:v>
+        <x:v>63</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="36" hidden="0" customHeight="1">
       <x:c r="A42" s="4" t="s">
-        <x:v>67</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="B42" s="5" t="s">
-        <x:v>68</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="C42" s="6" t="s">
         <x:v>7</x:v>
@@ -1216,10 +1217,10 @@
     </x:row>
     <x:row r="43" ht="24" hidden="0" customHeight="1">
       <x:c r="A43" s="4" t="s">
-        <x:v>69</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="B43" s="5" t="s">
-        <x:v>70</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="C43" s="6" t="s">
         <x:v>7</x:v>
@@ -1230,10 +1231,10 @@
     </x:row>
     <x:row r="44" ht="24" hidden="0" customHeight="1">
       <x:c r="A44" s="4" t="s">
-        <x:v>71</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="B44" s="5" t="s">
-        <x:v>72</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="C44" s="6" t="s">
         <x:v>7</x:v>
@@ -1244,10 +1245,10 @@
     </x:row>
     <x:row r="45" ht="36" hidden="0" customHeight="1">
       <x:c r="A45" s="4" t="s">
-        <x:v>73</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="B45" s="5" t="s">
-        <x:v>74</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="C45" s="6" t="str">
         <x:v>Done</x:v>
@@ -1258,10 +1259,10 @@
     </x:row>
     <x:row r="46" ht="24" hidden="0" customHeight="1">
       <x:c r="A46" s="4" t="s">
-        <x:v>75</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="B46" s="5" t="s">
-        <x:v>76</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="C46" s="6" t="str">
         <x:v>Done</x:v>
@@ -1272,10 +1273,10 @@
     </x:row>
     <x:row r="47" ht="36" hidden="0" customHeight="1">
       <x:c r="A47" s="4" t="s">
-        <x:v>77</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="B47" s="5" t="s">
-        <x:v>78</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="C47" s="6" t="str">
         <x:v>Done</x:v>
@@ -1286,7 +1287,7 @@
     </x:row>
     <x:row r="48" ht="15" customHeight="1">
       <x:c r="A48" s="14" t="s">
-        <x:v>79</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="B48" s="15"/>
       <x:c r="C48" s="16"/>
@@ -1294,10 +1295,10 @@
     </x:row>
     <x:row r="49" ht="60" hidden="0" customHeight="1">
       <x:c r="A49" s="4" t="s">
-        <x:v>80</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="B49" s="5" t="s">
-        <x:v>81</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="C49" s="6" t="str">
         <x:v>Done</x:v>
@@ -1308,51 +1309,53 @@
     </x:row>
     <x:row r="50" ht="15" customHeight="1">
       <x:c r="A50" s="4" t="s">
-        <x:v>82</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="B50" s="5" t="s">
-        <x:v>83</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="C50" s="6" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D50" s="7" t="s">
-        <x:v>84</x:v>
+        <x:v>81</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="15" customHeight="1">
       <x:c r="A51" s="4" t="s">
-        <x:v>85</x:v>
+        <x:v>82</x:v>
       </x:c>
       <x:c r="B51" s="5" t="s">
-        <x:v>86</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="C51" s="6" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D51" s="7" t="s">
-        <x:v>87</x:v>
+        <x:v>84</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="15" customHeight="1">
       <x:c r="A52" s="14" t="s">
-        <x:v>88</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="B52" s="15"/>
       <x:c r="C52" s="16"/>
       <x:c r="D52" s="17"/>
     </x:row>
-    <x:row r="53" ht="15" customHeight="1">
+    <x:row r="53" ht="24" hidden="0" customHeight="1">
       <x:c r="A53" s="8" t="s">
-        <x:v>89</x:v>
+        <x:v>86</x:v>
       </x:c>
       <x:c r="B53" s="9" t="s">
-        <x:v>90</x:v>
-      </x:c>
-      <x:c r="C53" s="10" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="D53" s="11"/>
+        <x:v>87</x:v>
+      </x:c>
+      <x:c r="C53" s="10" t="str">
+        <x:v>After launch</x:v>
+      </x:c>
+      <x:c r="D53" s="11" t="str">
+        <x:v>ANA-02 will be checked after operational deployment using live data. ANA-01 remains part of the production-scale validation.</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Mark KB-02 complete after Beta verification
</commit_message>
<xml_diff>
--- a/documentation/AITSM_Master_Checklist.xlsx
+++ b/documentation/AITSM_Master_Checklist.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Checklist" sheetId="1" r:id="Re3593da7c94647ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Checklist" sheetId="1" r:id="Ra495cd8b27af4d9f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1009,7 +1009,7 @@
       </x:c>
       <x:c r="D25" s="7"/>
     </x:row>
-    <x:row r="26" ht="24" hidden="0" customHeight="1">
+    <x:row r="26" ht="54" hidden="0" customHeight="1">
       <x:c r="A26" s="4" t="s">
         <x:v>37</x:v>
       </x:c>
@@ -1017,10 +1017,10 @@
         <x:v>Automatically detect recurring resolved issues and create a reviewable knowledge-base candidate after three similar occurrences.</x:v>
       </x:c>
       <x:c r="C26" s="6" t="str">
-        <x:v>Approved</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="D26" s="7" t="str">
-        <x:v>Approved design: store the suggested article, category, source ticket IDs, and occurrence count; require Super Admin review before publication.</x:v>
+        <x:v>Beta PR #27 verified on revision aitsm-beta-00083-zel. Three unique similar resolved tickets create a traceable candidate; Super Admin review is required before publication.</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="15" customHeight="1">

</xml_diff>

<commit_message>
Update master checklist for admin Beta fixes
</commit_message>
<xml_diff>
--- a/documentation/AITSM_Master_Checklist.xlsx
+++ b/documentation/AITSM_Master_Checklist.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Checklist" sheetId="1" r:id="Ra495cd8b27af4d9f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Checklist" sheetId="1" r:id="Rf1a99c3eeb1a4d21"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -844,7 +844,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="D10" s="7" t="str">
-        <x:v>Beta hardening completed: user-scoped counters now separate Open, In Progress, Resolved, Closed, and Total. Backend rules enforce Open → In Progress → Resolved → Closed and Resolved → In Progress. Resolution notes, history, and secure authenticated PNG/JPEG/WebP attachments are preserved.</x:v>
+        <x:v>Beta ticket lifecycle hardening remains complete. Admin dashboard ticket data now loads for regular Admin and Super Admin roles, Active and In Progress are counted separately, high-priority links use the authorized ticket feed, and Ticket Trend and Priority Distribution use the full paginated dataset.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" customHeight="1">
@@ -934,7 +934,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="D18" s="7" t="str">
-        <x:v>Includes two-device acceptance, revoked collector rejection, and dynamic-IP deduplication. The collector release remains HTTPS-hosted, SHA-256-pinned, scope-authorized, and free of localhost or machine-specific paths. Automated portability checks passed; a separate-PC install remains a manual acceptance test.</x:v>
+        <x:v>Includes two-device acceptance, revoked collector rejection, dynamic-IP deduplication, and scope authorization. Remove Collector now revokes and archives in one action for Admin and Super Admin; the collector and Diagnostics action disappear immediately while historical telemetry remains retained.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="15" customHeight="1">
@@ -977,7 +977,7 @@
       <x:c r="C22" s="16"/>
       <x:c r="D22" s="17"/>
     </x:row>
-    <x:row r="23" ht="15" customHeight="1">
+    <x:row r="23" ht="36" hidden="0" customHeight="1">
       <x:c r="A23" s="4" t="s">
         <x:v>32</x:v>
       </x:c>
@@ -987,7 +987,9 @@
       <x:c r="C23" s="6" t="s">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="D23" s="7"/>
+      <x:c r="D23" s="7" t="str">
+        <x:v>Inventory is the single device and asset view. Department is shown in the table, status filtering uses Online, Offline, and Stale, and the redundant Asset Management navigation and alphabetical status sorts were removed.</x:v>
+      </x:c>
     </x:row>
     <x:row r="24" ht="15" customHeight="1">
       <x:c r="A24" s="14" t="s">
@@ -1128,7 +1130,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="D35" s="18" t="str">
-        <x:v>111 automated tests passed. JavaScript syntax, dependency scanning with zero reported vulnerabilities, secret scanning, and Java/Kotlin and JavaScript CodeQL passed. Beta smoke tests returned HTTP 200. Manual acceptance remains for the two-role UI, browser attachment flow, forced-password flow, and separate-PC collector installation.</x:v>
+        <x:v>134 automated tests passed with zero failures or skips. JavaScript syntax, dependency scanning, secret scanning, and Java/Kotlin and JavaScript CodeQL passed. PR #29 deployed successfully to Beta revision aitsm-beta-00087-jil; the health endpoint returned status ok.</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="14.25" hidden="0" customHeight="1">
@@ -1176,7 +1178,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="D39" s="18" t="str">
-        <x:v>Six-issue Beta hardening is live on revision aitsm-beta-00052-waz from commit 569d2aa12b684ee9bdc4a084427430fedb4c0323. Three post-promotion health checks returned HTTP 200, legacy Gemini variables remain absent, and the prior revision is retained for rollback.</x:v>
+        <x:v>Protected GitHub-to-Google Cloud deployment remains operational. PR #29 passed tests and security scans, deployed through a no-traffic candidate, and promoted revision aitsm-beta-00087-jil to 100% of Beta traffic with a successful health check and rollback verification.</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="15" customHeight="1">

</xml_diff>

<commit_message>
Update analytics and collector checklist outcomes
</commit_message>
<xml_diff>
--- a/documentation/AITSM_Master_Checklist.xlsx
+++ b/documentation/AITSM_Master_Checklist.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Checklist" sheetId="1" r:id="Rf1a99c3eeb1a4d21"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Checklist" sheetId="1" r:id="Rbe41eb23fa454973"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -88,12 +88,6 @@
     <x:t xml:space="preserve">COL-19–20</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Collector update policy and possible macOS/Linux support.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">After launch</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">AI Assistance</x:t>
   </x:si>
   <x:si>
@@ -269,9 +263,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">ANA-01–02</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Validate analytics with production-scale data and define reports.</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -937,21 +928,23 @@
         <x:v>Includes two-device acceptance, revoked collector rejection, dynamic-IP deduplication, and scope authorization. Remove Collector now revokes and archives in one action for Admin and Super Admin; the collector and Diagnostics action disappear immediately while historical telemetry remains retained.</x:v>
       </x:c>
     </x:row>
-    <x:row r="19" ht="15" customHeight="1">
+    <x:row r="19" ht="84" hidden="0" customHeight="1">
       <x:c r="A19" s="4" t="s">
         <x:v>25</x:v>
       </x:c>
-      <x:c r="B19" s="5" t="s">
-        <x:v>26</x:v>
-      </x:c>
-      <x:c r="C19" s="6" t="s">
-        <x:v>27</x:v>
-      </x:c>
-      <x:c r="D19" s="7"/>
+      <x:c r="B19" s="5" t="str">
+        <x:v>Collector version/update policy and macOS/Linux feasibility decision.</x:v>
+      </x:c>
+      <x:c r="C19" s="6" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="D19" s="7" t="str">
+        <x:v>COL-19 completed: the portal reports current, update-available, unsupported, and legacy collector versions, with administrator-controlled update/repair installers pinned to the verified AITSM release. COL-20 completed as a production feasibility decision: Windows x64 remains the supported launch platform; macOS/Linux collectors are intentionally deferred until native service, secret-storage, signed-package, telemetry-parity, upgrade, and rollback requirements pass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="20" ht="15" customHeight="1">
       <x:c r="A20" s="14" t="s">
-        <x:v>28</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="B20" s="15"/>
       <x:c r="C20" s="16"/>
@@ -959,10 +952,10 @@
     </x:row>
     <x:row r="21" ht="24" customHeight="1">
       <x:c r="A21" s="4" t="s">
-        <x:v>29</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="B21" s="5" t="s">
-        <x:v>30</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="C21" s="6" t="s">
         <x:v>7</x:v>
@@ -971,7 +964,7 @@
     </x:row>
     <x:row r="22" ht="15" customHeight="1">
       <x:c r="A22" s="14" t="s">
-        <x:v>31</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="B22" s="15"/>
       <x:c r="C22" s="16"/>
@@ -979,10 +972,10 @@
     </x:row>
     <x:row r="23" ht="36" hidden="0" customHeight="1">
       <x:c r="A23" s="4" t="s">
-        <x:v>32</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="B23" s="5" t="s">
-        <x:v>33</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="C23" s="6" t="s">
         <x:v>7</x:v>
@@ -993,7 +986,7 @@
     </x:row>
     <x:row r="24" ht="15" customHeight="1">
       <x:c r="A24" s="14" t="s">
-        <x:v>34</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="B24" s="15"/>
       <x:c r="C24" s="16"/>
@@ -1001,10 +994,10 @@
     </x:row>
     <x:row r="25" ht="15" customHeight="1">
       <x:c r="A25" s="4" t="s">
-        <x:v>35</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="B25" s="5" t="s">
-        <x:v>36</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="C25" s="6" t="s">
         <x:v>7</x:v>
@@ -1013,7 +1006,7 @@
     </x:row>
     <x:row r="26" ht="54" hidden="0" customHeight="1">
       <x:c r="A26" s="4" t="s">
-        <x:v>37</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="B26" s="5" t="str">
         <x:v>Automatically detect recurring resolved issues and create a reviewable knowledge-base candidate after three similar occurrences.</x:v>
@@ -1027,10 +1020,10 @@
     </x:row>
     <x:row r="27" ht="15" customHeight="1">
       <x:c r="A27" s="4" t="s">
-        <x:v>38</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="B27" s="5" t="s">
-        <x:v>39</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="C27" s="6" t="s">
         <x:v>7</x:v>
@@ -1039,10 +1032,10 @@
     </x:row>
     <x:row r="28" ht="15" customHeight="1">
       <x:c r="A28" s="4" t="s">
-        <x:v>40</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="B28" s="5" t="s">
-        <x:v>41</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="C28" s="6" t="s">
         <x:v>7</x:v>
@@ -1051,10 +1044,10 @@
     </x:row>
     <x:row r="29" ht="24" hidden="0" customHeight="1">
       <x:c r="A29" s="4" t="s">
-        <x:v>42</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="B29" s="5" t="s">
-        <x:v>43</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="C29" s="6" t="str">
         <x:v>Done</x:v>
@@ -1065,7 +1058,7 @@
     </x:row>
     <x:row r="30" ht="15" customHeight="1">
       <x:c r="A30" s="14" t="s">
-        <x:v>44</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="B30" s="15"/>
       <x:c r="C30" s="16"/>
@@ -1073,10 +1066,10 @@
     </x:row>
     <x:row r="31" ht="15" customHeight="1">
       <x:c r="A31" s="4" t="s">
-        <x:v>45</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="B31" s="5" t="s">
-        <x:v>46</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="C31" s="6" t="s">
         <x:v>7</x:v>
@@ -1085,10 +1078,10 @@
     </x:row>
     <x:row r="32" ht="36" hidden="0" customHeight="1">
       <x:c r="A32" s="4" t="s">
-        <x:v>47</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="B32" s="5" t="s">
-        <x:v>48</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="C32" s="6" t="s">
         <x:v>7</x:v>
@@ -1099,10 +1092,10 @@
     </x:row>
     <x:row r="33" ht="72" hidden="0" customHeight="1">
       <x:c r="A33" s="4" t="s">
-        <x:v>49</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="B33" s="5" t="s">
-        <x:v>50</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="C33" s="6" t="str">
         <x:v>Done</x:v>
@@ -1113,29 +1106,29 @@
     </x:row>
     <x:row r="34" ht="15" customHeight="1">
       <x:c r="A34" s="14" t="s">
-        <x:v>51</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="B34" s="15"/>
       <x:c r="C34" s="16"/>
       <x:c r="D34" s="19"/>
     </x:row>
-    <x:row r="35" ht="92" customHeight="1">
+    <x:row r="35" ht="48" hidden="0" customHeight="1">
       <x:c r="A35" s="4" t="s">
-        <x:v>52</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="B35" s="5" t="s">
-        <x:v>53</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="C35" s="6" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D35" s="18" t="str">
-        <x:v>134 automated tests passed with zero failures or skips. JavaScript syntax, dependency scanning, secret scanning, and Java/Kotlin and JavaScript CodeQL passed. PR #29 deployed successfully to Beta revision aitsm-beta-00087-jil; the health endpoint returned status ok.</x:v>
+        <x:v>140 automated tests passed with zero failures or skips. JavaScript syntax, dependency scanning, secret scanning, and Java/Kotlin and JavaScript CodeQL passed. PRs #32 and #33 deployed successfully to Beta revision aitsm-beta-00093-ror; the health endpoint returned status ok.</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="14.25" hidden="0" customHeight="1">
       <x:c r="A36" s="4" t="s">
-        <x:v>54</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="B36" s="5" t="str">
         <x:v>Browser-level end-to-end regression pass.</x:v>
@@ -1149,7 +1142,7 @@
     </x:row>
     <x:row r="37" ht="15" customHeight="1">
       <x:c r="A37" s="14" t="s">
-        <x:v>55</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="B37" s="15"/>
       <x:c r="C37" s="16"/>
@@ -1157,33 +1150,33 @@
     </x:row>
     <x:row r="38" ht="15" customHeight="1">
       <x:c r="A38" s="4" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="B38" s="5" t="s">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="C38" s="6" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="D38" s="18"/>
+    </x:row>
+    <x:row r="39" ht="48" hidden="0" customHeight="1">
+      <x:c r="A39" s="4" t="s">
         <x:v>56</x:v>
       </x:c>
-      <x:c r="B38" s="5" t="s">
+      <x:c r="B39" s="5" t="s">
         <x:v>57</x:v>
       </x:c>
-      <x:c r="C38" s="6" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="D38" s="18"/>
-    </x:row>
-    <x:row r="39" ht="76" hidden="0" customHeight="1">
-      <x:c r="A39" s="4" t="s">
-        <x:v>58</x:v>
-      </x:c>
-      <x:c r="B39" s="5" t="s">
-        <x:v>59</x:v>
-      </x:c>
       <x:c r="C39" s="6" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D39" s="18" t="str">
-        <x:v>Protected GitHub-to-Google Cloud deployment remains operational. PR #29 passed tests and security scans, deployed through a no-traffic candidate, and promoted revision aitsm-beta-00087-jil to 100% of Beta traffic with a successful health check and rollback verification.</x:v>
+        <x:v>Protected GitHub-to-Google Cloud deployment remains operational. PRs #32 and #33 passed tests and security scans, deployed through a no-traffic candidate, and promoted revision aitsm-beta-00093-ror to 100% of Beta traffic with a successful health check and rollback verification.</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="15" customHeight="1">
       <x:c r="A40" s="14" t="s">
-        <x:v>60</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="B40" s="15"/>
       <x:c r="C40" s="16"/>
@@ -1191,24 +1184,24 @@
     </x:row>
     <x:row r="41" ht="15" customHeight="1">
       <x:c r="A41" s="4" t="s">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="B41" s="5" t="s">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="C41" s="6" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="D41" s="18" t="s">
         <x:v>61</x:v>
-      </x:c>
-      <x:c r="B41" s="5" t="s">
-        <x:v>62</x:v>
-      </x:c>
-      <x:c r="C41" s="6" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="D41" s="18" t="s">
-        <x:v>63</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="36" hidden="0" customHeight="1">
       <x:c r="A42" s="4" t="s">
-        <x:v>64</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="B42" s="5" t="s">
-        <x:v>65</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="C42" s="6" t="s">
         <x:v>7</x:v>
@@ -1219,10 +1212,10 @@
     </x:row>
     <x:row r="43" ht="24" hidden="0" customHeight="1">
       <x:c r="A43" s="4" t="s">
-        <x:v>66</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="B43" s="5" t="s">
-        <x:v>67</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="C43" s="6" t="s">
         <x:v>7</x:v>
@@ -1233,10 +1226,10 @@
     </x:row>
     <x:row r="44" ht="24" hidden="0" customHeight="1">
       <x:c r="A44" s="4" t="s">
-        <x:v>68</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="B44" s="5" t="s">
-        <x:v>69</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="C44" s="6" t="s">
         <x:v>7</x:v>
@@ -1247,10 +1240,10 @@
     </x:row>
     <x:row r="45" ht="36" hidden="0" customHeight="1">
       <x:c r="A45" s="4" t="s">
-        <x:v>70</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="B45" s="5" t="s">
-        <x:v>71</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="C45" s="6" t="str">
         <x:v>Done</x:v>
@@ -1261,10 +1254,10 @@
     </x:row>
     <x:row r="46" ht="24" hidden="0" customHeight="1">
       <x:c r="A46" s="4" t="s">
-        <x:v>72</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="B46" s="5" t="s">
-        <x:v>73</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="C46" s="6" t="str">
         <x:v>Done</x:v>
@@ -1275,10 +1268,10 @@
     </x:row>
     <x:row r="47" ht="36" hidden="0" customHeight="1">
       <x:c r="A47" s="4" t="s">
-        <x:v>74</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="B47" s="5" t="s">
-        <x:v>75</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="C47" s="6" t="str">
         <x:v>Done</x:v>
@@ -1289,7 +1282,7 @@
     </x:row>
     <x:row r="48" ht="15" customHeight="1">
       <x:c r="A48" s="14" t="s">
-        <x:v>76</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="B48" s="15"/>
       <x:c r="C48" s="16"/>
@@ -1297,10 +1290,10 @@
     </x:row>
     <x:row r="49" ht="60" hidden="0" customHeight="1">
       <x:c r="A49" s="4" t="s">
-        <x:v>77</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="B49" s="5" t="s">
-        <x:v>78</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="C49" s="6" t="str">
         <x:v>Done</x:v>
@@ -1311,52 +1304,52 @@
     </x:row>
     <x:row r="50" ht="15" customHeight="1">
       <x:c r="A50" s="4" t="s">
+        <x:v>77</x:v>
+      </x:c>
+      <x:c r="B50" s="5" t="s">
+        <x:v>78</x:v>
+      </x:c>
+      <x:c r="C50" s="6" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="D50" s="7" t="s">
         <x:v>79</x:v>
-      </x:c>
-      <x:c r="B50" s="5" t="s">
-        <x:v>80</x:v>
-      </x:c>
-      <x:c r="C50" s="6" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="D50" s="7" t="s">
-        <x:v>81</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="15" customHeight="1">
       <x:c r="A51" s="4" t="s">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="B51" s="5" t="s">
+        <x:v>81</x:v>
+      </x:c>
+      <x:c r="C51" s="6" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="D51" s="7" t="s">
         <x:v>82</x:v>
-      </x:c>
-      <x:c r="B51" s="5" t="s">
-        <x:v>83</x:v>
-      </x:c>
-      <x:c r="C51" s="6" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="D51" s="7" t="s">
-        <x:v>84</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="15" customHeight="1">
       <x:c r="A52" s="14" t="s">
-        <x:v>85</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="B52" s="15"/>
       <x:c r="C52" s="16"/>
       <x:c r="D52" s="17"/>
     </x:row>
-    <x:row r="53" ht="24" hidden="0" customHeight="1">
+    <x:row r="53" ht="72" hidden="0" customHeight="1">
       <x:c r="A53" s="8" t="s">
-        <x:v>86</x:v>
-      </x:c>
-      <x:c r="B53" s="9" t="s">
-        <x:v>87</x:v>
+        <x:v>84</x:v>
+      </x:c>
+      <x:c r="B53" s="9" t="str">
+        <x:v>Validate analytics and provide protected operational reporting export.</x:v>
       </x:c>
       <x:c r="C53" s="10" t="str">
-        <x:v>After launch</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="D53" s="11" t="str">
-        <x:v>ANA-02 will be checked after operational deployment using live data. ANA-01 remains part of the production-scale validation.</x:v>
+        <x:v>ANA-01 completed through the user-confirmed dashboard and chart validation. ANA-02 completed with an administrator-only, reauthentication-protected, audited CSV export containing ticket classification, status, assignment, timestamps, and SLA risk fields while excluding descriptions and authentication data. Verified on Beta revision aitsm-beta-00093-ror.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>